<commit_message>
Update Velocity distribution of an object in its life history.xlsx
</commit_message>
<xml_diff>
--- a/Analysis/Velocity distribution of an object in its life history.xlsx
+++ b/Analysis/Velocity distribution of an object in its life history.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Documents\GitHub\article\Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64E6386E-1EF5-41EB-B8C9-5A3452DB02BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{919BDD15-A9FE-42A6-A31B-ED538298447F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -151,7 +151,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Length distribution of an object in its life history</a:t>
+              <a:t>Velocity distribution of an object in its life history</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1748,7 +1748,7 @@
               <a:rPr lang="en-US" sz="1800" b="0" i="0" baseline="0">
                 <a:effectLst/>
               </a:rPr>
-              <a:t>Length distribution of an object in its life history</a:t>
+              <a:t>Velocity distribution of an object in its life history</a:t>
             </a:r>
             <a:endParaRPr lang="en-US">
               <a:effectLst/>

</xml_diff>